<commit_message>
dados: D09 registra revisão do artigo e pertinência das colunas
</commit_message>
<xml_diff>
--- a/data-raw/D09_tilapia_sensorial/tilapia_sensorial_para_revisao.xlsx
+++ b/data-raw/D09_tilapia_sensorial/tilapia_sensorial_para_revisao.xlsx
@@ -3317,7 +3317,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="65" customWidth="1" min="1" max="1"/>
@@ -3414,10 +3414,26 @@
         </is>
       </c>
     </row>
+    <row r="15" ht="70" customHeight="1">
+      <c r="A15" s="16" t="inlineStr">
+        <is>
+          <t>Pendência registrada em 11/10/2026: o professor consultará o artigo para esclarecer a escala e as medidas. Depois, avaliar quais colunas são pertinentes à análise e justificar eventual retirada. A coluna específica ainda não foi indicada; os dados completos permanecem preservados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="60" customHeight="1">
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>Após ler o artigo: explicação das medidas e decisão sobre quais colunas usar</t>
+        </is>
+      </c>
+      <c r="B17" s="17" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A13:B13"/>
     <mergeCell ref="A11:B11"/>
+    <mergeCell ref="A15:B15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>